<commit_message>
feat: shared mask subgraph, zoning, road frontage
</commit_message>
<xml_diff>
--- a/docs/module_list.xlsx
+++ b/docs/module_list.xlsx
@@ -893,7 +893,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
+          <t>/Game/StarterContent/Shapes/Shape_Cylinder.Shape_Cylinder</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Placeholders/SM_Cube.SM_Cube</t>
+          <t>/Game/Meshes/Placeholders/SM_Cone.SM_Cone</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat: graph parameters for frontage, lot size and density
</commit_message>
<xml_diff>
--- a/docs/module_list.xlsx
+++ b/docs/module_list.xlsx
@@ -777,7 +777,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Block_Mid.SM_Residential_Block_Mid</t>
+          <t>/Game/StarterContent/Shapes/Shape_Cube.Shape_Cube</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -835,7 +835,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Terrace.SM_Residential_Terrace</t>
+          <t>/Game/StarterContent/Shapes/Shape_Wedge_A.Shape_Wedge_A</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -951,7 +951,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Industrial_Processing.SM_Industrial_Processing</t>
+          <t>/Game/StarterContent/Shapes/Shape_Tube.Shape_Tube</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Service_Utility_Block.SM_Service_Utility_Block</t>
+          <t>/Game/StarterContent/Shapes/Shape_Sphere.Shape_Sphere</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">

</xml_diff>